<commit_message>
docs(tesis): documentación Scrum del Proyecto APT al 29-10-2026
- Cierre del Sprint 3 (16-10): Release v1.3.0, Review y Retro; Backlog,
  Scrumboard, Burndown e Impedimentos en v1.2. HU-12 no aceptada.
- Sprint 4 (S11-S12) hasta el día 9: Planning, Backlog, Scrumboard,
  Burndown e Impedimentos (IMP-16 e IMP-17).
- Daily Meeting #01 a #58 (archivo renombrado a "S1 a S12").
- Product Backlog v1.6 y planilla de seguimiento al 29-10.
- Presentación de avance (29-10-2026).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tesis/00 - Listado de documentos - Seguimiento.xlsx
+++ b/tesis/00 - Listado de documentos - Seguimiento.xlsx
@@ -503,7 +503,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>EvangelicApp · Proyecto APT 2026-2 — Seguimiento de documentos Scrum (actualizado al 08-10-2026, semana S9)</t>
+          <t>EvangelicApp · Proyecto APT 2026-2 — Seguimiento de documentos Scrum (actualizado al 29-10-2026, semana S12)</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Documento vivo: v1.4 al 05-10 (Planning del Sprint 3)</t>
+          <t>Documento vivo: v1.6 al 19-10 (Planning del Sprint 4)</t>
         </is>
       </c>
     </row>
@@ -1102,17 +1102,17 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>S1 a S9</t>
+          <t>S1 a S12</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>S1–S9</t>
+          <t>S1–S12</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>08-10-2026</t>
+          <t>29-10-2026</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>12 - Daily Meeting (S1 a S9).docx</t>
+          <t>12 - Daily Meeting (S1 a S12).docx</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>43 Daily; se actualiza a diario</t>
+          <t>58 Daily; se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>12 - Daily Meeting (S1 a S9).docx</t>
+          <t>12 - Daily Meeting (S1 a S12).docx</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>12 - Daily Meeting (S1 a S9).docx</t>
+          <t>12 - Daily Meeting (S1 a S12).docx</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -1903,12 +1903,12 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>08-10-2026</t>
+          <t>16-10-2026</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Planning, Backlog, Scrumboard, Burndown e Impedimentos al día 4 de 10; Release, Review y Retro el 16-10</t>
+          <t>Sprint cerrado el 16-10: Release v1.3.0, Review y Retro (velocidad 21/26; HU-12 no aceptada)</t>
         </is>
       </c>
     </row>
@@ -1948,22 +1948,22 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>29-10-2026</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6. Sprint 4 - QA de seguridad, k6 y Realtime (S11-S12)/</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Según Carta Gantt</t>
+          <t>Planning, Backlog, Scrumboard, Burndown e Impedimentos al día 9 de 10; Release v1.4.0, Review y Retro el 30-10</t>
         </is>
       </c>
     </row>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sprint 3: RLS multi-tenant y staging  ← HOY (08-10)</t>
+          <t>Sprint 3: RLS multi-tenant y staging</t>
         </is>
       </c>
     </row>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sprint 4 · Documentación e informe final</t>
+          <t>Sprint 4 (cierre el 30-10) · Documentación e informe final  ← HOY (29-10)</t>
         </is>
       </c>
     </row>

</xml_diff>